<commit_message>
add stock data free query support
</commit_message>
<xml_diff>
--- a/TMIS数据自由查询参数模板_v5.1.xlsx
+++ b/TMIS数据自由查询参数模板_v5.1.xlsx
@@ -10,6 +10,7 @@
     <sheet name="收入参数" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="支出参数" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="退库参数" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="库存参数" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1141,4 +1142,248 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:W2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>文件名称</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>是否追加日期</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>保留原文件名</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>报表库选择</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>报表类型</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>起始日期</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>终止日期</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>国库选择</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>辖属标志</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>国库属性</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>预算级次</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>会计科目</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>会计账户名称</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>计划单列市/县/乡</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>展示范围</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>金额单位</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>分序时</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>分地区</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>分国库属性</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>分预算级次</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>分会计科目</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>分会计账户</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>是否展示同比</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>库存自由查询</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1 -- 报表库</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>3 -- 月</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>202601</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>202603</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0 -- 全辖</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>0 -- 全部</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>271,272,273</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0 -- 不含</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>1 -- 下级</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>0 -- 元</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>